<commit_message>
Split supplier letters into individually named files
Each of the eleven letters now lives in its own file under
egypt-jan-2027/Письма/, named so the filename states the recipient and
the purpose, and opens with a header table giving КОМУ, ОТДЕЛ, ТЕМА,
КОГДА and ЗАЧЕМ plus a checklist of what a complete reply must contain.

Also:
- Rebuilt 04-PISMA-I-KONTAKTY.md around a summary table mapping letter
  number to recipient, department, subject line and send date.
- Added a Hilton Luxor room-block letter (previously only a note), so
  the set covers both river options.
- Added a "Реестр писем" tracking sheet to Бюджет_Египет_2027.xlsx for
  sent/answered/reference-number status.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KQFm1d6HbwvN6nT4uerjN3
</commit_message>
<xml_diff>
--- a/egypt-jan-2027/Бюджет_Египет_2027.xlsx
+++ b/egypt-jan-2027/Бюджет_Египет_2027.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Расчёт" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Билеты" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Статусы услуг" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сценарии" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реестр писем" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Расчёт" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Билеты" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Статусы услуг" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сценарии" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +69,11 @@
       <i val="1"/>
       <color rgb="00C00000"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -124,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -162,6 +168,12 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -527,6 +539,538 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>РЕЕСТР ПИСЕМ · Египет 23–30 января 2027 · La Royal Event</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Жёлтые столбцы заполняете вы по мере отправки. Ответ без номера заявки статус не меняет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Название письма</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Кому</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="inlineStr">
+        <is>
+          <t>Отдел</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Тема письма</t>
+        </is>
+      </c>
+      <c r="F4" s="25" t="inlineStr">
+        <is>
+          <t>Когда отправить</t>
+        </is>
+      </c>
+      <c r="G4" s="25" t="inlineStr">
+        <is>
+          <t>Дата отправки</t>
+        </is>
+      </c>
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>Дата ответа</t>
+        </is>
+      </c>
+      <c r="I4" s="25" t="inlineStr">
+        <is>
+          <t>Номер заявки</t>
+        </is>
+      </c>
+      <c r="J4" s="25" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Запрос полного фрахта судна</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Судовые операторы: Sun Boat III, Oberoi, дахабии</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Charters &amp; Private Groups</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>Full charter enquiry — 14–16 guests, single occupancy, 23–30 January 2027</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>СЕГОДНЯ</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Запрос наземных услуг</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Принимающая компания, 2–3 кандидата</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Incoming / MICE</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Ground services RFP — private group 14–16, Cairo / Luxor / Aswan, 23–30 January 2027</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>в течение 3 дней</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Ночное посещение Гизы</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Подрядчик спецдоступов</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Permits</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>Private night access, Giza — 18 persons, 24 January 2027</t>
+        </is>
+      </c>
+      <c r="F7" s="26" t="inlineStr">
+        <is>
+          <t>СЕГОДНЯ</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Приватное посещение Филе и показ</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Подрядчик спецдоступов</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>Permits</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Philae — private visit and private Sound &amp; Light session, 28 January 2027, 18 pax</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>после ответов судов</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Гала-ужин и ответ по номерам</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Mandarin Oriental, Old Cataract, Асуан</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Events &amp; Catering, НЕ Reservations</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Private gala dinner enquiry — 18 guests, 29 January 2027</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>в течение 3 дней</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Блок номеров в Каире</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Marriott Mena House</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Group Sales / Sales &amp; Events</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Group block enquiry — 18 rooms, mainly single occupancy, 23–25 January 2027</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>после выбора судна</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Блок номеров в Луксоре</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>Hilton Luxor Resort &amp; Spa</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Group Reservations</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Group block enquiry — 18 rooms, mainly single occupancy, 25–26 January 2027</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>только для варианта II</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Блок номеров в Асуане</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Mövenpick Resort Aswan</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Group Reservations</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Group block enquiry — 18 rooms single occupancy, 29–30 January 2027</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>после выбора судна</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Приватный полёт на шаре</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Лицензированный оператор шаров, Луксор</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Reservations</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Private balloon flight enquiry — 16–18 passengers, Luxor, 26 January 2027</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>ноябрь 2026</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Внутренние перелёты на группу</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>EgyptAir, Nile Air или через DMC</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>Group Desk</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Group booking enquiry — 18 passengers, CAI–LXR 25 Jan 2027 and ASW–CAI 30 Jan 2027</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>в течение 3 дней</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Предложение и вопросы</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>КЛИЕНТ</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Египет, 23–30 января 2027: предложение и вопросы для бронирования</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr">
+        <is>
+          <t>СЕГОДНЯ</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>не отправлено</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1350,7 +1894,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1771,7 +2315,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2373,7 +2917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>